<commit_message>
Cost by Tier: subtotal row after each plan block
A shaded TOTAL row now closes each plan's four tier rows, giving
enrolled headcount, Onyx per month and per year, employees per
month and per year, and the combined worst case for everyone on
that plan. A blank spacer separates the blocks.

The subtotal rows are excluded from every lookup and roll-up: their
plan label carries a TOTAL suffix, so the Combined tab's SUMIFS and
SUMPRODUCT skip them and nothing double counts.

553 formulas, zero errors; all cells re-verified and every toggle
re-tested.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E1Hoi5T9BmzS6cxcPMES4F
</commit_message>
<xml_diff>
--- a/deliverables/Onyx_Angle_Questco_Cost_Model.xlsx
+++ b/deliverables/Onyx_Angle_Questco_Cost_Model.xlsx
@@ -19,8 +19,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'By Employee'!$A$4:$M$19</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Cost by Tier'!$A$4:$S$16</definedName>
-    <definedName function="false" hidden="false" name="CostKey" vbProcedure="false">'Cost by Tier'!$T$5:$T$16</definedName>
+    <definedName function="false" hidden="false" name="CostKey" vbProcedure="false">'Cost by Tier'!$T$5:$T$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="317">
   <si>
     <t xml:space="preserve">Onyx Accounting Group, LLC - Angle Health + Questco</t>
   </si>
@@ -344,6 +343,21 @@
   </si>
   <si>
     <t xml:space="preserve">Row key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG HDHP 3400/5000  -  TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All tiers counted in totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL ROW - not a lookup key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG TRAD 2000/4000  -  TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG TRAD 1000/2000  -  TOTAL</t>
   </si>
   <si>
     <t xml:space="preserve">HSA funding is deliberately not modeled. On the HDHP 3400/5000 an employee can pay part of that worst case with pretax dollars, so the real cost is lower - but by an amount only the employee controls.</t>
@@ -1230,7 +1244,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="79">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1491,7 +1505,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1500,6 +1514,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1548,7 +1570,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1568,22 +1590,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF808080"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1669,10 +1675,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -2660,7 +2662,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -3073,241 +3075,129 @@
         <v>ANG HDHP 3400/5000|FAM</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="65" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="34" t="n">
+        <f aca="false">SUM(E5:E8)</f>
+        <v>4</v>
+      </c>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="66" t="n">
+        <f aca="false">SUM(L5:L8)</f>
+        <v>2041.5</v>
+      </c>
+      <c r="M9" s="67" t="n">
+        <f aca="false">SUM(M5:M8)</f>
+        <v>24498</v>
+      </c>
+      <c r="N9" s="66" t="n">
+        <f aca="false">SUM(N5:N8)</f>
+        <v>2041.5</v>
+      </c>
+      <c r="O9" s="67" t="n">
+        <f aca="false">SUM(O5:O8)</f>
+        <v>24498</v>
+      </c>
+      <c r="P9" s="33"/>
+      <c r="Q9" s="33"/>
+      <c r="R9" s="33"/>
+      <c r="S9" s="67" t="n">
+        <f aca="false">SUMPRODUCT($S5:$S8,$E5:$E8)</f>
+        <v>59498</v>
+      </c>
+      <c r="T9" s="68" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="28" t="str">
-        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C9,Contributions!$B$11:$B$14,0))</f>
+      <c r="D11" s="28" t="str">
+        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C11,Contributions!$B$11:$B$14,0))</f>
         <v>Yes</v>
       </c>
-      <c r="E9" s="11" t="n">
-        <f aca="false">IF($D9&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C9,Contributions!$E$26:$E$30,"Yes"))</f>
+      <c r="E11" s="11" t="n">
+        <f aca="false">IF($D11&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C11,Contributions!$E$26:$E$30,"Yes"))</f>
         <v>1</v>
       </c>
-      <c r="F9" s="15" t="n">
-        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A9,'Angle Plans'!$A$5:$A$7,0),MATCH($C9,'Angle Plans'!$L$4:$O$4,0))</f>
+      <c r="F11" s="15" t="n">
+        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0),MATCH($C11,'Angle Plans'!$L$4:$O$4,0))</f>
         <v>492.11</v>
       </c>
-      <c r="G9" s="15" t="n">
-        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C9,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C9,Contributions!$B$11:$B$14,0))*$F9)</f>
+      <c r="G11" s="15" t="n">
+        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C11,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C11,Contributions!$B$11:$B$14,0))*$F11)</f>
         <v>246.055</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H11" s="15" t="n">
         <f aca="false">Contributions!$C$20</f>
         <v>219.515</v>
       </c>
-      <c r="I9" s="47" t="n">
-        <f aca="false">MIN($F9,MAX($G9,$H9))</f>
+      <c r="I11" s="47" t="n">
+        <f aca="false">MIN($F11,MAX($G11,$H11))</f>
         <v>246.055</v>
       </c>
-      <c r="J9" s="47" t="n">
-        <f aca="false">$F9-$I9</f>
+      <c r="J11" s="47" t="n">
+        <f aca="false">$F11-$I11</f>
         <v>246.055</v>
       </c>
-      <c r="K9" s="48" t="n">
-        <f aca="false">IF($F9=0,0,$I9/$F9)</f>
-        <v>0.5</v>
-      </c>
-      <c r="L9" s="47" t="n">
-        <f aca="false">$I9*$E9</f>
-        <v>246.055</v>
-      </c>
-      <c r="M9" s="25" t="n">
-        <f aca="false">$L9*12</f>
-        <v>2952.66</v>
-      </c>
-      <c r="N9" s="47" t="n">
-        <f aca="false">$J9*$E9</f>
-        <v>246.055</v>
-      </c>
-      <c r="O9" s="25" t="n">
-        <f aca="false">$N9*12</f>
-        <v>2952.66</v>
-      </c>
-      <c r="P9" s="25" t="n">
-        <f aca="false">$J9*12</f>
-        <v>2952.66</v>
-      </c>
-      <c r="Q9" s="49" t="n">
-        <f aca="false">IF($C9="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A9,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A9,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>2000</v>
-      </c>
-      <c r="R9" s="49" t="n">
-        <f aca="false">IF($C9="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A9,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A9,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>4000</v>
-      </c>
-      <c r="S9" s="50" t="n">
-        <f aca="false">$P9+$R9</f>
-        <v>6952.66</v>
-      </c>
-      <c r="T9" s="51" t="str">
-        <f aca="false">$A9&amp;"|"&amp;$C9</f>
-        <v>ANG TRAD 2000/4000|EE</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="52" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="53" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="54" t="str">
-        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C10,Contributions!$B$11:$B$14,0))</f>
-        <v>Yes</v>
-      </c>
-      <c r="E10" s="53" t="n">
-        <f aca="false">IF($D10&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C10,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>1</v>
-      </c>
-      <c r="F10" s="55" t="n">
-        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A10,'Angle Plans'!$A$5:$A$7,0),MATCH($C10,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>1033.43</v>
-      </c>
-      <c r="G10" s="55" t="n">
-        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C10,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C10,Contributions!$B$11:$B$14,0))*$F10)</f>
-        <v>516.715</v>
-      </c>
-      <c r="H10" s="55" t="n">
-        <f aca="false">Contributions!$C$20</f>
-        <v>219.515</v>
-      </c>
-      <c r="I10" s="56" t="n">
-        <f aca="false">MIN($F10,MAX($G10,$H10))</f>
-        <v>516.715</v>
-      </c>
-      <c r="J10" s="56" t="n">
-        <f aca="false">$F10-$I10</f>
-        <v>516.715</v>
-      </c>
-      <c r="K10" s="57" t="n">
-        <f aca="false">IF($F10=0,0,$I10/$F10)</f>
-        <v>0.5</v>
-      </c>
-      <c r="L10" s="56" t="n">
-        <f aca="false">$I10*$E10</f>
-        <v>516.715</v>
-      </c>
-      <c r="M10" s="58" t="n">
-        <f aca="false">$L10*12</f>
-        <v>6200.58</v>
-      </c>
-      <c r="N10" s="56" t="n">
-        <f aca="false">$J10*$E10</f>
-        <v>516.715</v>
-      </c>
-      <c r="O10" s="58" t="n">
-        <f aca="false">$N10*12</f>
-        <v>6200.58</v>
-      </c>
-      <c r="P10" s="58" t="n">
-        <f aca="false">$J10*12</f>
-        <v>6200.58</v>
-      </c>
-      <c r="Q10" s="59" t="n">
-        <f aca="false">IF($C10="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A10,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A10,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>4000</v>
-      </c>
-      <c r="R10" s="59" t="n">
-        <f aca="false">IF($C10="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A10,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A10,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>8000</v>
-      </c>
-      <c r="S10" s="60" t="n">
-        <f aca="false">$P10+$R10</f>
-        <v>14200.58</v>
-      </c>
-      <c r="T10" s="51" t="str">
-        <f aca="false">$A10&amp;"|"&amp;$C10</f>
-        <v>ANG TRAD 2000/4000|ES</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="31" t="str">
-        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C11,Contributions!$B$11:$B$14,0))</f>
-        <v>No</v>
-      </c>
-      <c r="E11" s="18" t="n">
-        <f aca="false">IF($D11&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C11,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="21" t="n">
-        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0),MATCH($C11,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>934.01</v>
-      </c>
-      <c r="G11" s="21" t="n">
-        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C11,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C11,Contributions!$B$11:$B$14,0))*$F11)</f>
-        <v>467.005</v>
-      </c>
-      <c r="H11" s="21" t="n">
-        <f aca="false">Contributions!$C$20</f>
-        <v>219.515</v>
-      </c>
-      <c r="I11" s="61" t="n">
-        <f aca="false">MIN($F11,MAX($G11,$H11))</f>
-        <v>467.005</v>
-      </c>
-      <c r="J11" s="61" t="n">
-        <f aca="false">$F11-$I11</f>
-        <v>467.005</v>
-      </c>
-      <c r="K11" s="62" t="n">
+      <c r="K11" s="48" t="n">
         <f aca="false">IF($F11=0,0,$I11/$F11)</f>
         <v>0.5</v>
       </c>
-      <c r="L11" s="61" t="n">
+      <c r="L11" s="47" t="n">
         <f aca="false">$I11*$E11</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="63" t="n">
+        <v>246.055</v>
+      </c>
+      <c r="M11" s="25" t="n">
         <f aca="false">$L11*12</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="61" t="n">
+        <v>2952.66</v>
+      </c>
+      <c r="N11" s="47" t="n">
         <f aca="false">$J11*$E11</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="63" t="n">
+        <v>246.055</v>
+      </c>
+      <c r="O11" s="25" t="n">
         <f aca="false">$N11*12</f>
-        <v>0</v>
-      </c>
-      <c r="P11" s="63" t="n">
+        <v>2952.66</v>
+      </c>
+      <c r="P11" s="25" t="n">
         <f aca="false">$J11*12</f>
-        <v>5604.06</v>
-      </c>
-      <c r="Q11" s="64" t="n">
+        <v>2952.66</v>
+      </c>
+      <c r="Q11" s="49" t="n">
         <f aca="false">IF($C11="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>2000</v>
+      </c>
+      <c r="R11" s="49" t="n">
+        <f aca="false">IF($C11="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)))</f>
         <v>4000</v>
       </c>
-      <c r="R11" s="64" t="n">
-        <f aca="false">IF($C11="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A11,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>8000</v>
-      </c>
-      <c r="S11" s="63" t="n">
+      <c r="S11" s="50" t="n">
         <f aca="false">$P11+$R11</f>
-        <v>13604.06</v>
+        <v>6952.66</v>
       </c>
       <c r="T11" s="51" t="str">
         <f aca="false">$A11&amp;"|"&amp;$C11</f>
-        <v>ANG TRAD 2000/4000|EC</v>
+        <v>ANG TRAD 2000/4000|EE</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3315,10 +3205,10 @@
         <v>71</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D12" s="54" t="str">
         <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C12,Contributions!$B$11:$B$14,0))</f>
@@ -3326,15 +3216,15 @@
       </c>
       <c r="E12" s="53" t="n">
         <f aca="false">IF($D12&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C12,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="55" t="n">
         <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A12,'Angle Plans'!$A$5:$A$7,0),MATCH($C12,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>1525.54</v>
+        <v>1033.43</v>
       </c>
       <c r="G12" s="55" t="n">
         <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C12,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C12,Contributions!$B$11:$B$14,0))*$F12)</f>
-        <v>762.77</v>
+        <v>516.715</v>
       </c>
       <c r="H12" s="55" t="n">
         <f aca="false">Contributions!$C$20</f>
@@ -3342,11 +3232,11 @@
       </c>
       <c r="I12" s="56" t="n">
         <f aca="false">MIN($F12,MAX($G12,$H12))</f>
-        <v>762.77</v>
+        <v>516.715</v>
       </c>
       <c r="J12" s="56" t="n">
         <f aca="false">$F12-$I12</f>
-        <v>762.77</v>
+        <v>516.715</v>
       </c>
       <c r="K12" s="57" t="n">
         <f aca="false">IF($F12=0,0,$I12/$F12)</f>
@@ -3354,23 +3244,23 @@
       </c>
       <c r="L12" s="56" t="n">
         <f aca="false">$I12*$E12</f>
-        <v>1525.54</v>
+        <v>516.715</v>
       </c>
       <c r="M12" s="58" t="n">
         <f aca="false">$L12*12</f>
-        <v>18306.48</v>
+        <v>6200.58</v>
       </c>
       <c r="N12" s="56" t="n">
         <f aca="false">$J12*$E12</f>
-        <v>1525.54</v>
+        <v>516.715</v>
       </c>
       <c r="O12" s="58" t="n">
         <f aca="false">$N12*12</f>
-        <v>18306.48</v>
+        <v>6200.58</v>
       </c>
       <c r="P12" s="58" t="n">
         <f aca="false">$J12*12</f>
-        <v>9153.24</v>
+        <v>6200.58</v>
       </c>
       <c r="Q12" s="59" t="n">
         <f aca="false">IF($C12="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A12,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A12,'Angle Plans'!$A$5:$A$7,0)))</f>
@@ -3382,101 +3272,101 @@
       </c>
       <c r="S12" s="60" t="n">
         <f aca="false">$P12+$R12</f>
-        <v>17153.24</v>
+        <v>14200.58</v>
       </c>
       <c r="T12" s="51" t="str">
         <f aca="false">$A12&amp;"|"&amp;$C12</f>
-        <v>ANG TRAD 2000/4000|FAM</v>
+        <v>ANG TRAD 2000/4000|ES</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="28" t="str">
+      <c r="A13" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="31" t="str">
         <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C13,Contributions!$B$11:$B$14,0))</f>
-        <v>Yes</v>
-      </c>
-      <c r="E13" s="11" t="n">
+        <v>No</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <f aca="false">IF($D13&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C13,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>1</v>
-      </c>
-      <c r="F13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="21" t="n">
         <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A13,'Angle Plans'!$A$5:$A$7,0),MATCH($C13,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>546.33</v>
-      </c>
-      <c r="G13" s="15" t="n">
+        <v>934.01</v>
+      </c>
+      <c r="G13" s="21" t="n">
         <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C13,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C13,Contributions!$B$11:$B$14,0))*$F13)</f>
-        <v>273.165</v>
-      </c>
-      <c r="H13" s="15" t="n">
+        <v>467.005</v>
+      </c>
+      <c r="H13" s="21" t="n">
         <f aca="false">Contributions!$C$20</f>
         <v>219.515</v>
       </c>
-      <c r="I13" s="47" t="n">
+      <c r="I13" s="61" t="n">
         <f aca="false">MIN($F13,MAX($G13,$H13))</f>
-        <v>273.165</v>
-      </c>
-      <c r="J13" s="47" t="n">
+        <v>467.005</v>
+      </c>
+      <c r="J13" s="61" t="n">
         <f aca="false">$F13-$I13</f>
-        <v>273.165</v>
-      </c>
-      <c r="K13" s="48" t="n">
+        <v>467.005</v>
+      </c>
+      <c r="K13" s="62" t="n">
         <f aca="false">IF($F13=0,0,$I13/$F13)</f>
         <v>0.5</v>
       </c>
-      <c r="L13" s="47" t="n">
+      <c r="L13" s="61" t="n">
         <f aca="false">$I13*$E13</f>
-        <v>273.165</v>
-      </c>
-      <c r="M13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="63" t="n">
         <f aca="false">$L13*12</f>
-        <v>3277.98</v>
-      </c>
-      <c r="N13" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="61" t="n">
         <f aca="false">$J13*$E13</f>
-        <v>273.165</v>
-      </c>
-      <c r="O13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="63" t="n">
         <f aca="false">$N13*12</f>
-        <v>3277.98</v>
-      </c>
-      <c r="P13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="63" t="n">
         <f aca="false">$J13*12</f>
-        <v>3277.98</v>
-      </c>
-      <c r="Q13" s="49" t="n">
+        <v>5604.06</v>
+      </c>
+      <c r="Q13" s="64" t="n">
         <f aca="false">IF($C13="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A13,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A13,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>1000</v>
-      </c>
-      <c r="R13" s="49" t="n">
+        <v>4000</v>
+      </c>
+      <c r="R13" s="64" t="n">
         <f aca="false">IF($C13="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A13,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A13,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>2000</v>
-      </c>
-      <c r="S13" s="50" t="n">
+        <v>8000</v>
+      </c>
+      <c r="S13" s="63" t="n">
         <f aca="false">$P13+$R13</f>
-        <v>5277.98</v>
+        <v>13604.06</v>
       </c>
       <c r="T13" s="51" t="str">
         <f aca="false">$A13&amp;"|"&amp;$C13</f>
-        <v>ANG TRAD 1000/2000|EE</v>
+        <v>ANG TRAD 2000/4000|EC</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="52" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D14" s="54" t="str">
         <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C14,Contributions!$B$11:$B$14,0))</f>
@@ -3484,15 +3374,15 @@
       </c>
       <c r="E14" s="53" t="n">
         <f aca="false">IF($D14&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C14,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="55" t="n">
         <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A14,'Angle Plans'!$A$5:$A$7,0),MATCH($C14,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>1147.29</v>
+        <v>1525.54</v>
       </c>
       <c r="G14" s="55" t="n">
         <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C14,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C14,Contributions!$B$11:$B$14,0))*$F14)</f>
-        <v>573.645</v>
+        <v>762.77</v>
       </c>
       <c r="H14" s="55" t="n">
         <f aca="false">Contributions!$C$20</f>
@@ -3500,11 +3390,11 @@
       </c>
       <c r="I14" s="56" t="n">
         <f aca="false">MIN($F14,MAX($G14,$H14))</f>
-        <v>573.645</v>
+        <v>762.77</v>
       </c>
       <c r="J14" s="56" t="n">
         <f aca="false">$F14-$I14</f>
-        <v>573.645</v>
+        <v>762.77</v>
       </c>
       <c r="K14" s="57" t="n">
         <f aca="false">IF($F14=0,0,$I14/$F14)</f>
@@ -3512,211 +3402,460 @@
       </c>
       <c r="L14" s="56" t="n">
         <f aca="false">$I14*$E14</f>
-        <v>573.645</v>
+        <v>1525.54</v>
       </c>
       <c r="M14" s="58" t="n">
         <f aca="false">$L14*12</f>
-        <v>6883.74</v>
+        <v>18306.48</v>
       </c>
       <c r="N14" s="56" t="n">
         <f aca="false">$J14*$E14</f>
-        <v>573.645</v>
+        <v>1525.54</v>
       </c>
       <c r="O14" s="58" t="n">
         <f aca="false">$N14*12</f>
-        <v>6883.74</v>
+        <v>18306.48</v>
       </c>
       <c r="P14" s="58" t="n">
         <f aca="false">$J14*12</f>
-        <v>6883.74</v>
+        <v>9153.24</v>
       </c>
       <c r="Q14" s="59" t="n">
         <f aca="false">IF($C14="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A14,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A14,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="R14" s="59" t="n">
         <f aca="false">IF($C14="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A14,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A14,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>4000</v>
+        <v>8000</v>
       </c>
       <c r="S14" s="60" t="n">
         <f aca="false">$P14+$R14</f>
-        <v>10883.74</v>
+        <v>17153.24</v>
       </c>
       <c r="T14" s="51" t="str">
         <f aca="false">$A14&amp;"|"&amp;$C14</f>
-        <v>ANG TRAD 1000/2000|ES</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+        <v>ANG TRAD 2000/4000|FAM</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="B15" s="65" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34" t="n">
+        <f aca="false">SUM(E11:E14)</f>
+        <v>4</v>
+      </c>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="66" t="n">
+        <f aca="false">SUM(L11:L14)</f>
+        <v>2288.31</v>
+      </c>
+      <c r="M15" s="67" t="n">
+        <f aca="false">SUM(M11:M14)</f>
+        <v>27459.72</v>
+      </c>
+      <c r="N15" s="66" t="n">
+        <f aca="false">SUM(N11:N14)</f>
+        <v>2288.31</v>
+      </c>
+      <c r="O15" s="67" t="n">
+        <f aca="false">SUM(O11:O14)</f>
+        <v>27459.72</v>
+      </c>
+      <c r="P15" s="33"/>
+      <c r="Q15" s="33"/>
+      <c r="R15" s="33"/>
+      <c r="S15" s="67" t="n">
+        <f aca="false">SUMPRODUCT($S11:$S14,$E11:$E14)</f>
+        <v>55459.72</v>
+      </c>
+      <c r="T15" s="68" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="31" t="str">
-        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C15,Contributions!$B$11:$B$14,0))</f>
-        <v>No</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <f aca="false">IF($D15&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C15,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="21" t="n">
-        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A15,'Angle Plans'!$A$5:$A$7,0),MATCH($C15,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>1038.02</v>
-      </c>
-      <c r="G15" s="21" t="n">
-        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C15,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C15,Contributions!$B$11:$B$14,0))*$F15)</f>
-        <v>519.01</v>
-      </c>
-      <c r="H15" s="21" t="n">
+      <c r="B17" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="28" t="str">
+        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C17,Contributions!$B$11:$B$14,0))</f>
+        <v>Yes</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <f aca="false">IF($D17&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C17,Contributions!$E$26:$E$30,"Yes"))</f>
+        <v>1</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A17,'Angle Plans'!$A$5:$A$7,0),MATCH($C17,'Angle Plans'!$L$4:$O$4,0))</f>
+        <v>546.33</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C17,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C17,Contributions!$B$11:$B$14,0))*$F17)</f>
+        <v>273.165</v>
+      </c>
+      <c r="H17" s="15" t="n">
         <f aca="false">Contributions!$C$20</f>
         <v>219.515</v>
       </c>
-      <c r="I15" s="61" t="n">
-        <f aca="false">MIN($F15,MAX($G15,$H15))</f>
-        <v>519.01</v>
-      </c>
-      <c r="J15" s="61" t="n">
-        <f aca="false">$F15-$I15</f>
-        <v>519.01</v>
-      </c>
-      <c r="K15" s="62" t="n">
-        <f aca="false">IF($F15=0,0,$I15/$F15)</f>
+      <c r="I17" s="47" t="n">
+        <f aca="false">MIN($F17,MAX($G17,$H17))</f>
+        <v>273.165</v>
+      </c>
+      <c r="J17" s="47" t="n">
+        <f aca="false">$F17-$I17</f>
+        <v>273.165</v>
+      </c>
+      <c r="K17" s="48" t="n">
+        <f aca="false">IF($F17=0,0,$I17/$F17)</f>
         <v>0.5</v>
       </c>
-      <c r="L15" s="61" t="n">
-        <f aca="false">$I15*$E15</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="63" t="n">
-        <f aca="false">$L15*12</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="61" t="n">
-        <f aca="false">$J15*$E15</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="63" t="n">
-        <f aca="false">$N15*12</f>
-        <v>0</v>
-      </c>
-      <c r="P15" s="63" t="n">
-        <f aca="false">$J15*12</f>
-        <v>6228.12</v>
-      </c>
-      <c r="Q15" s="64" t="n">
-        <f aca="false">IF($C15="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A15,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A15,'Angle Plans'!$A$5:$A$7,0)))</f>
+      <c r="L17" s="47" t="n">
+        <f aca="false">$I17*$E17</f>
+        <v>273.165</v>
+      </c>
+      <c r="M17" s="25" t="n">
+        <f aca="false">$L17*12</f>
+        <v>3277.98</v>
+      </c>
+      <c r="N17" s="47" t="n">
+        <f aca="false">$J17*$E17</f>
+        <v>273.165</v>
+      </c>
+      <c r="O17" s="25" t="n">
+        <f aca="false">$N17*12</f>
+        <v>3277.98</v>
+      </c>
+      <c r="P17" s="25" t="n">
+        <f aca="false">$J17*12</f>
+        <v>3277.98</v>
+      </c>
+      <c r="Q17" s="49" t="n">
+        <f aca="false">IF($C17="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A17,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A17,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>1000</v>
+      </c>
+      <c r="R17" s="49" t="n">
+        <f aca="false">IF($C17="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A17,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A17,'Angle Plans'!$A$5:$A$7,0)))</f>
         <v>2000</v>
       </c>
-      <c r="R15" s="64" t="n">
-        <f aca="false">IF($C15="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A15,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A15,'Angle Plans'!$A$5:$A$7,0)))</f>
-        <v>4000</v>
-      </c>
-      <c r="S15" s="63" t="n">
-        <f aca="false">$P15+$R15</f>
-        <v>10228.12</v>
-      </c>
-      <c r="T15" s="51" t="str">
-        <f aca="false">$A15&amp;"|"&amp;$C15</f>
-        <v>ANG TRAD 1000/2000|EC</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="52" t="s">
+      <c r="S17" s="50" t="n">
+        <f aca="false">$P17+$R17</f>
+        <v>5277.98</v>
+      </c>
+      <c r="T17" s="51" t="str">
+        <f aca="false">$A17&amp;"|"&amp;$C17</f>
+        <v>ANG TRAD 1000/2000|EE</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="52" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="54" t="str">
-        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C16,Contributions!$B$11:$B$14,0))</f>
+      <c r="B18" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="54" t="str">
+        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C18,Contributions!$B$11:$B$14,0))</f>
         <v>Yes</v>
       </c>
-      <c r="E16" s="53" t="n">
-        <f aca="false">IF($D16&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C16,Contributions!$E$26:$E$30,"Yes"))</f>
-        <v>2</v>
-      </c>
-      <c r="F16" s="55" t="n">
-        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A16,'Angle Plans'!$A$5:$A$7,0),MATCH($C16,'Angle Plans'!$L$4:$O$4,0))</f>
-        <v>1693.61</v>
-      </c>
-      <c r="G16" s="55" t="n">
-        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C16,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C16,Contributions!$B$11:$B$14,0))*$F16)</f>
-        <v>846.805</v>
-      </c>
-      <c r="H16" s="55" t="n">
+      <c r="E18" s="53" t="n">
+        <f aca="false">IF($D18&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C18,Contributions!$E$26:$E$30,"Yes"))</f>
+        <v>1</v>
+      </c>
+      <c r="F18" s="55" t="n">
+        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A18,'Angle Plans'!$A$5:$A$7,0),MATCH($C18,'Angle Plans'!$L$4:$O$4,0))</f>
+        <v>1147.29</v>
+      </c>
+      <c r="G18" s="55" t="n">
+        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C18,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C18,Contributions!$B$11:$B$14,0))*$F18)</f>
+        <v>573.645</v>
+      </c>
+      <c r="H18" s="55" t="n">
         <f aca="false">Contributions!$C$20</f>
         <v>219.515</v>
       </c>
-      <c r="I16" s="56" t="n">
-        <f aca="false">MIN($F16,MAX($G16,$H16))</f>
+      <c r="I18" s="56" t="n">
+        <f aca="false">MIN($F18,MAX($G18,$H18))</f>
+        <v>573.645</v>
+      </c>
+      <c r="J18" s="56" t="n">
+        <f aca="false">$F18-$I18</f>
+        <v>573.645</v>
+      </c>
+      <c r="K18" s="57" t="n">
+        <f aca="false">IF($F18=0,0,$I18/$F18)</f>
+        <v>0.5</v>
+      </c>
+      <c r="L18" s="56" t="n">
+        <f aca="false">$I18*$E18</f>
+        <v>573.645</v>
+      </c>
+      <c r="M18" s="58" t="n">
+        <f aca="false">$L18*12</f>
+        <v>6883.74</v>
+      </c>
+      <c r="N18" s="56" t="n">
+        <f aca="false">$J18*$E18</f>
+        <v>573.645</v>
+      </c>
+      <c r="O18" s="58" t="n">
+        <f aca="false">$N18*12</f>
+        <v>6883.74</v>
+      </c>
+      <c r="P18" s="58" t="n">
+        <f aca="false">$J18*12</f>
+        <v>6883.74</v>
+      </c>
+      <c r="Q18" s="59" t="n">
+        <f aca="false">IF($C18="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A18,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A18,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>2000</v>
+      </c>
+      <c r="R18" s="59" t="n">
+        <f aca="false">IF($C18="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A18,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A18,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>4000</v>
+      </c>
+      <c r="S18" s="60" t="n">
+        <f aca="false">$P18+$R18</f>
+        <v>10883.74</v>
+      </c>
+      <c r="T18" s="51" t="str">
+        <f aca="false">$A18&amp;"|"&amp;$C18</f>
+        <v>ANG TRAD 1000/2000|ES</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="31" t="str">
+        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C19,Contributions!$B$11:$B$14,0))</f>
+        <v>No</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <f aca="false">IF($D19&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C19,Contributions!$E$26:$E$30,"Yes"))</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A19,'Angle Plans'!$A$5:$A$7,0),MATCH($C19,'Angle Plans'!$L$4:$O$4,0))</f>
+        <v>1038.02</v>
+      </c>
+      <c r="G19" s="21" t="n">
+        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C19,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C19,Contributions!$B$11:$B$14,0))*$F19)</f>
+        <v>519.01</v>
+      </c>
+      <c r="H19" s="21" t="n">
+        <f aca="false">Contributions!$C$20</f>
+        <v>219.515</v>
+      </c>
+      <c r="I19" s="61" t="n">
+        <f aca="false">MIN($F19,MAX($G19,$H19))</f>
+        <v>519.01</v>
+      </c>
+      <c r="J19" s="61" t="n">
+        <f aca="false">$F19-$I19</f>
+        <v>519.01</v>
+      </c>
+      <c r="K19" s="62" t="n">
+        <f aca="false">IF($F19=0,0,$I19/$F19)</f>
+        <v>0.5</v>
+      </c>
+      <c r="L19" s="61" t="n">
+        <f aca="false">$I19*$E19</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="63" t="n">
+        <f aca="false">$L19*12</f>
+        <v>0</v>
+      </c>
+      <c r="N19" s="61" t="n">
+        <f aca="false">$J19*$E19</f>
+        <v>0</v>
+      </c>
+      <c r="O19" s="63" t="n">
+        <f aca="false">$N19*12</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="63" t="n">
+        <f aca="false">$J19*12</f>
+        <v>6228.12</v>
+      </c>
+      <c r="Q19" s="64" t="n">
+        <f aca="false">IF($C19="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A19,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A19,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>2000</v>
+      </c>
+      <c r="R19" s="64" t="n">
+        <f aca="false">IF($C19="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A19,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A19,'Angle Plans'!$A$5:$A$7,0)))</f>
+        <v>4000</v>
+      </c>
+      <c r="S19" s="63" t="n">
+        <f aca="false">$P19+$R19</f>
+        <v>10228.12</v>
+      </c>
+      <c r="T19" s="51" t="str">
+        <f aca="false">$A19&amp;"|"&amp;$C19</f>
+        <v>ANG TRAD 1000/2000|EC</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" s="54" t="str">
+        <f aca="false">INDEX(Contributions!$C$11:$C$14,MATCH($C20,Contributions!$B$11:$B$14,0))</f>
+        <v>Yes</v>
+      </c>
+      <c r="E20" s="53" t="n">
+        <f aca="false">IF($D20&lt;&gt;"Yes",0,COUNTIFS(Contributions!$D$26:$D$30,$C20,Contributions!$E$26:$E$30,"Yes"))</f>
+        <v>2</v>
+      </c>
+      <c r="F20" s="55" t="n">
+        <f aca="false">INDEX('Angle Plans'!$L$5:$O$7,MATCH($A20,'Angle Plans'!$A$5:$A$7,0),MATCH($C20,'Angle Plans'!$L$4:$O$4,0))</f>
+        <v>1693.61</v>
+      </c>
+      <c r="G20" s="55" t="n">
+        <f aca="false">IF(Contributions!$C$6="Fixed dollars",INDEX(Contributions!$E$11:$E$14,MATCH($C20,Contributions!$B$11:$B$14,0)),INDEX(Contributions!$D$11:$D$14,MATCH($C20,Contributions!$B$11:$B$14,0))*$F20)</f>
         <v>846.805</v>
       </c>
-      <c r="J16" s="56" t="n">
-        <f aca="false">$F16-$I16</f>
+      <c r="H20" s="55" t="n">
+        <f aca="false">Contributions!$C$20</f>
+        <v>219.515</v>
+      </c>
+      <c r="I20" s="56" t="n">
+        <f aca="false">MIN($F20,MAX($G20,$H20))</f>
         <v>846.805</v>
       </c>
-      <c r="K16" s="57" t="n">
-        <f aca="false">IF($F16=0,0,$I16/$F16)</f>
+      <c r="J20" s="56" t="n">
+        <f aca="false">$F20-$I20</f>
+        <v>846.805</v>
+      </c>
+      <c r="K20" s="57" t="n">
+        <f aca="false">IF($F20=0,0,$I20/$F20)</f>
         <v>0.5</v>
       </c>
-      <c r="L16" s="56" t="n">
-        <f aca="false">$I16*$E16</f>
+      <c r="L20" s="56" t="n">
+        <f aca="false">$I20*$E20</f>
         <v>1693.61</v>
       </c>
-      <c r="M16" s="58" t="n">
-        <f aca="false">$L16*12</f>
+      <c r="M20" s="58" t="n">
+        <f aca="false">$L20*12</f>
         <v>20323.32</v>
       </c>
-      <c r="N16" s="56" t="n">
-        <f aca="false">$J16*$E16</f>
+      <c r="N20" s="56" t="n">
+        <f aca="false">$J20*$E20</f>
         <v>1693.61</v>
       </c>
-      <c r="O16" s="58" t="n">
-        <f aca="false">$N16*12</f>
+      <c r="O20" s="58" t="n">
+        <f aca="false">$N20*12</f>
         <v>20323.32</v>
       </c>
-      <c r="P16" s="58" t="n">
-        <f aca="false">$J16*12</f>
+      <c r="P20" s="58" t="n">
+        <f aca="false">$J20*12</f>
         <v>10161.66</v>
       </c>
-      <c r="Q16" s="59" t="n">
-        <f aca="false">IF($C16="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A16,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A16,'Angle Plans'!$A$5:$A$7,0)))</f>
+      <c r="Q20" s="59" t="n">
+        <f aca="false">IF($C20="EE",INDEX('Angle Plans'!$C$5:$C$7,MATCH($A20,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$D$5:$D$7,MATCH($A20,'Angle Plans'!$A$5:$A$7,0)))</f>
         <v>2000</v>
       </c>
-      <c r="R16" s="59" t="n">
-        <f aca="false">IF($C16="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A16,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A16,'Angle Plans'!$A$5:$A$7,0)))</f>
+      <c r="R20" s="59" t="n">
+        <f aca="false">IF($C20="EE",INDEX('Angle Plans'!$E$5:$E$7,MATCH($A20,'Angle Plans'!$A$5:$A$7,0)),INDEX('Angle Plans'!$F$5:$F$7,MATCH($A20,'Angle Plans'!$A$5:$A$7,0)))</f>
         <v>4000</v>
       </c>
-      <c r="S16" s="60" t="n">
-        <f aca="false">$P16+$R16</f>
+      <c r="S20" s="60" t="n">
+        <f aca="false">$P20+$R20</f>
         <v>14161.66</v>
       </c>
-      <c r="T16" s="51" t="str">
-        <f aca="false">$A16&amp;"|"&amp;$C16</f>
+      <c r="T20" s="51" t="str">
+        <f aca="false">$A20&amp;"|"&amp;$C20</f>
         <v>ANG TRAD 1000/2000|FAM</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="65" t="s">
         <v>105</v>
       </c>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="34" t="n">
+        <f aca="false">SUM(E17:E20)</f>
+        <v>4</v>
+      </c>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="66" t="n">
+        <f aca="false">SUM(L17:L20)</f>
+        <v>2540.42</v>
+      </c>
+      <c r="M21" s="67" t="n">
+        <f aca="false">SUM(M17:M20)</f>
+        <v>30485.04</v>
+      </c>
+      <c r="N21" s="66" t="n">
+        <f aca="false">SUM(N17:N20)</f>
+        <v>2540.42</v>
+      </c>
+      <c r="O21" s="67" t="n">
+        <f aca="false">SUM(O17:O20)</f>
+        <v>30485.04</v>
+      </c>
+      <c r="P21" s="33"/>
+      <c r="Q21" s="33"/>
+      <c r="R21" s="33"/>
+      <c r="S21" s="67" t="n">
+        <f aca="false">SUMPRODUCT($S17:$S20,$E17:$E20)</f>
+        <v>44485.04</v>
+      </c>
+      <c r="T21" s="68" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>110</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:S16"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3724,7 +3863,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3752,22 +3890,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -3796,7 +3934,7 @@
         <v>9</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>89</v>
@@ -3805,22 +3943,22 @@
         <v>90</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3846,15 +3984,15 @@
         <v>Yes</v>
       </c>
       <c r="G7" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H7" s="47" t="n">
-        <f aca="false">IF(OR($B7&lt;&gt;"Yes",$F7&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0)))</f>
+        <f aca="false">IF(OR($B7&lt;&gt;"Yes",$F7&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0)))</f>
         <v>680.5</v>
       </c>
       <c r="I7" s="47" t="n">
-        <f aca="false">IF(OR($B7&lt;&gt;"Yes",$F7&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0)))</f>
+        <f aca="false">IF(OR($B7&lt;&gt;"Yes",$F7&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0)))</f>
         <v>680.5</v>
       </c>
       <c r="J7" s="24" t="n">
@@ -3897,15 +4035,15 @@
         <v>Yes</v>
       </c>
       <c r="G8" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>439.03</v>
       </c>
       <c r="H8" s="47" t="n">
-        <f aca="false">IF(OR($B8&lt;&gt;"Yes",$F8&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0)))</f>
+        <f aca="false">IF(OR($B8&lt;&gt;"Yes",$F8&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0)))</f>
         <v>219.515</v>
       </c>
       <c r="I8" s="47" t="n">
-        <f aca="false">IF(OR($B8&lt;&gt;"Yes",$F8&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0)))</f>
+        <f aca="false">IF(OR($B8&lt;&gt;"Yes",$F8&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0)))</f>
         <v>219.515</v>
       </c>
       <c r="J8" s="24" t="n">
@@ -3948,15 +4086,15 @@
         <v>Yes</v>
       </c>
       <c r="G9" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H9" s="47" t="n">
-        <f aca="false">IF(OR($B9&lt;&gt;"Yes",$F9&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0)))</f>
+        <f aca="false">IF(OR($B9&lt;&gt;"Yes",$F9&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0)))</f>
         <v>680.5</v>
       </c>
       <c r="I9" s="47" t="n">
-        <f aca="false">IF(OR($B9&lt;&gt;"Yes",$F9&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0)))</f>
+        <f aca="false">IF(OR($B9&lt;&gt;"Yes",$F9&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0)))</f>
         <v>680.5</v>
       </c>
       <c r="J9" s="24" t="n">
@@ -3999,15 +4137,15 @@
         <v>Yes</v>
       </c>
       <c r="G10" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>921.97</v>
       </c>
       <c r="H10" s="47" t="n">
-        <f aca="false">IF(OR($B10&lt;&gt;"Yes",$F10&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0)))</f>
+        <f aca="false">IF(OR($B10&lt;&gt;"Yes",$F10&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0)))</f>
         <v>460.985</v>
       </c>
       <c r="I10" s="47" t="n">
-        <f aca="false">IF(OR($B10&lt;&gt;"Yes",$F10&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0)))</f>
+        <f aca="false">IF(OR($B10&lt;&gt;"Yes",$F10&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0)))</f>
         <v>460.985</v>
       </c>
       <c r="J10" s="24" t="n">
@@ -4050,18 +4188,18 @@
         <v>Yes</v>
       </c>
       <c r="G11" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H11" s="56" t="n">
-        <f aca="false">IF(OR($B11&lt;&gt;"Yes",$F11&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0)))</f>
+        <f aca="false">IF(OR($B11&lt;&gt;"Yes",$F11&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0)))</f>
         <v>0</v>
       </c>
       <c r="I11" s="56" t="n">
-        <f aca="false">IF(OR($B11&lt;&gt;"Yes",$F11&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0)))</f>
+        <f aca="false">IF(OR($B11&lt;&gt;"Yes",$F11&lt;&gt;"Yes"),0,INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0)))</f>
         <v>0</v>
       </c>
-      <c r="J11" s="65" t="n">
+      <c r="J11" s="69" t="n">
         <f aca="false">$H11+$I11</f>
         <v>0</v>
       </c>
@@ -4080,7 +4218,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B12" s="34" t="str">
         <f aca="false">COUNTIF(B7:B11,"Yes")&amp;" enrolled"</f>
@@ -4118,7 +4256,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="66" t="n">
@@ -4128,7 +4266,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="67" t="n">
@@ -4138,7 +4276,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="47" t="n">
@@ -4148,7 +4286,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="25" t="n">
@@ -4158,12 +4296,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -4204,12 +4342,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4235,13 +4373,13 @@
         <v>90</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K4" s="9" t="s">
         <v>100</v>
@@ -4250,7 +4388,7 @@
         <v>101</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,35 +4409,35 @@
         <v>66</v>
       </c>
       <c r="F5" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G5" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H5" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="I5" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="J5" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>8166</v>
       </c>
       <c r="K5" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>6800</v>
       </c>
       <c r="L5" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M5" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
+      <c r="M5" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>18166</v>
       </c>
     </row>
@@ -4321,35 +4459,35 @@
         <v>71</v>
       </c>
       <c r="F6" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G6" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>1525.54</v>
       </c>
       <c r="H6" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="I6" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="J6" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>9153.24</v>
       </c>
       <c r="K6" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>4000</v>
       </c>
       <c r="L6" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M6" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
+      <c r="M6" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>17153.24</v>
       </c>
     </row>
@@ -4371,35 +4509,35 @@
         <v>78</v>
       </c>
       <c r="F7" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G7" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>1693.61</v>
       </c>
       <c r="H7" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="I7" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="J7" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>10161.66</v>
       </c>
       <c r="K7" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>2000</v>
       </c>
       <c r="L7" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M7" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
+      <c r="M7" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>14161.66</v>
       </c>
     </row>
@@ -4421,35 +4559,35 @@
         <v>66</v>
       </c>
       <c r="F8" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G8" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>439.03</v>
       </c>
       <c r="H8" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>219.515</v>
       </c>
       <c r="I8" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>219.515</v>
       </c>
       <c r="J8" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>2634.18</v>
       </c>
       <c r="K8" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>3400</v>
       </c>
       <c r="L8" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>5000</v>
       </c>
-      <c r="M8" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
+      <c r="M8" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>7634.18</v>
       </c>
     </row>
@@ -4471,35 +4609,35 @@
         <v>71</v>
       </c>
       <c r="F9" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G9" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>492.11</v>
       </c>
       <c r="H9" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>246.055</v>
       </c>
       <c r="I9" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>246.055</v>
       </c>
       <c r="J9" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>2952.66</v>
       </c>
       <c r="K9" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>2000</v>
       </c>
       <c r="L9" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M9" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
+      <c r="M9" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>6952.66</v>
       </c>
     </row>
@@ -4521,35 +4659,35 @@
         <v>78</v>
       </c>
       <c r="F10" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G10" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>546.33</v>
       </c>
       <c r="H10" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>273.165</v>
       </c>
       <c r="I10" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>273.165</v>
       </c>
       <c r="J10" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>3277.98</v>
       </c>
       <c r="K10" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>1000</v>
       </c>
       <c r="L10" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>2000</v>
       </c>
-      <c r="M10" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
+      <c r="M10" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>5277.98</v>
       </c>
     </row>
@@ -4571,35 +4709,35 @@
         <v>66</v>
       </c>
       <c r="F11" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G11" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H11" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="I11" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="J11" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>8166</v>
       </c>
       <c r="K11" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>6800</v>
       </c>
       <c r="L11" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M11" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
+      <c r="M11" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>18166</v>
       </c>
     </row>
@@ -4621,35 +4759,35 @@
         <v>71</v>
       </c>
       <c r="F12" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G12" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>1525.54</v>
       </c>
       <c r="H12" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="I12" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="J12" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>9153.24</v>
       </c>
       <c r="K12" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>4000</v>
       </c>
       <c r="L12" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M12" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
+      <c r="M12" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>17153.24</v>
       </c>
     </row>
@@ -4671,35 +4809,35 @@
         <v>78</v>
       </c>
       <c r="F13" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G13" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>1693.61</v>
       </c>
       <c r="H13" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="I13" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="J13" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>10161.66</v>
       </c>
       <c r="K13" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>2000</v>
       </c>
       <c r="L13" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M13" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
+      <c r="M13" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>14161.66</v>
       </c>
     </row>
@@ -4721,35 +4859,35 @@
         <v>66</v>
       </c>
       <c r="F14" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G14" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>921.97</v>
       </c>
       <c r="H14" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>460.985</v>
       </c>
       <c r="I14" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>460.985</v>
       </c>
       <c r="J14" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>5531.82</v>
       </c>
       <c r="K14" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>6800</v>
       </c>
       <c r="L14" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M14" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
+      <c r="M14" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>15531.82</v>
       </c>
     </row>
@@ -4771,35 +4909,35 @@
         <v>71</v>
       </c>
       <c r="F15" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G15" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>1033.43</v>
       </c>
       <c r="H15" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>516.715</v>
       </c>
       <c r="I15" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>516.715</v>
       </c>
       <c r="J15" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>6200.58</v>
       </c>
       <c r="K15" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>4000</v>
       </c>
       <c r="L15" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M15" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
+      <c r="M15" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>14200.58</v>
       </c>
     </row>
@@ -4821,35 +4959,35 @@
         <v>78</v>
       </c>
       <c r="F16" s="28" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G16" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>1147.29</v>
       </c>
       <c r="H16" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>573.645</v>
       </c>
       <c r="I16" s="15" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>573.645</v>
       </c>
       <c r="J16" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>6883.74</v>
       </c>
       <c r="K16" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>2000</v>
       </c>
       <c r="L16" s="49" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M16" s="68" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
+      <c r="M16" s="70" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>10883.74</v>
       </c>
     </row>
@@ -4871,35 +5009,35 @@
         <v>66</v>
       </c>
       <c r="F17" s="54" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G17" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>1361</v>
       </c>
       <c r="H17" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="I17" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>680.5</v>
       </c>
       <c r="J17" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>8166</v>
       </c>
       <c r="K17" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>6800</v>
       </c>
       <c r="L17" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M17" s="69" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
+      <c r="M17" s="71" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>18166</v>
       </c>
     </row>
@@ -4921,35 +5059,35 @@
         <v>71</v>
       </c>
       <c r="F18" s="54" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G18" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>1525.54</v>
       </c>
       <c r="H18" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="I18" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>762.77</v>
       </c>
       <c r="J18" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>9153.24</v>
       </c>
       <c r="K18" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>4000</v>
       </c>
       <c r="L18" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M18" s="69" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
+      <c r="M18" s="71" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>17153.24</v>
       </c>
     </row>
@@ -4971,35 +5109,35 @@
         <v>78</v>
       </c>
       <c r="F19" s="54" t="str">
-        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$D$5:$D$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>Yes</v>
       </c>
       <c r="G19" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$F$5:$F$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>1693.61</v>
       </c>
       <c r="H19" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$I$5:$I$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="I19" s="55" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$J$5:$J$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>846.805</v>
       </c>
       <c r="J19" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$P$5:$P$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>10161.66</v>
       </c>
       <c r="K19" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$Q$5:$Q$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>2000</v>
       </c>
       <c r="L19" s="59" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+        <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M19" s="69" t="n">
-        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$16,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
+      <c r="M19" s="71" t="n">
+        <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>14161.66</v>
       </c>
     </row>
@@ -5035,17 +5173,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -5057,25 +5195,25 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>38</v>
@@ -5083,10 +5221,10 @@
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B6" s="70" t="s">
-        <v>139</v>
+        <v>143</v>
+      </c>
+      <c r="B6" s="72" t="s">
+        <v>144</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>117</v>
@@ -5094,8 +5232,8 @@
       <c r="D6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="71" t="s">
-        <v>140</v>
+      <c r="E6" s="73" t="s">
+        <v>145</v>
       </c>
       <c r="F6" s="47" t="n">
         <f aca="false">G6/12</f>
@@ -5106,22 +5244,22 @@
         <v>7020</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B7" s="70" t="s">
-        <v>143</v>
+        <v>147</v>
+      </c>
+      <c r="B7" s="72" t="s">
+        <v>148</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>1402.13</v>
       </c>
       <c r="D7" s="7"/>
-      <c r="E7" s="71" t="s">
-        <v>140</v>
+      <c r="E7" s="73" t="s">
+        <v>145</v>
       </c>
       <c r="F7" s="47" t="n">
         <f aca="false">G7/12</f>
@@ -5132,15 +5270,15 @@
         <v>1402.13</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="70" t="s">
-        <v>143</v>
+        <v>150</v>
+      </c>
+      <c r="B8" s="72" t="s">
+        <v>148</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>420</v>
@@ -5158,12 +5296,12 @@
         <v>0</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
@@ -5181,28 +5319,28 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="B10" s="70" t="s">
-        <v>149</v>
+        <v>153</v>
+      </c>
+      <c r="B10" s="72" t="s">
+        <v>154</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
-      <c r="G10" s="72" t="n">
+      <c r="G10" s="74" t="n">
         <v>1000</v>
       </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -5214,19 +5352,19 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>38</v>
@@ -5234,13 +5372,13 @@
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="70" t="s">
-        <v>155</v>
+      <c r="C15" s="72" t="s">
+        <v>160</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>46.25</v>
@@ -5250,18 +5388,18 @@
         <v>555</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="70" t="s">
-        <v>158</v>
+      <c r="C16" s="72" t="s">
+        <v>163</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>159.09</v>
@@ -5271,18 +5409,18 @@
         <v>1909.08</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="70" t="s">
-        <v>161</v>
+      <c r="C17" s="72" t="s">
+        <v>166</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>126.74</v>
@@ -5292,12 +5430,12 @@
         <v>0</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="33"/>
@@ -5313,12 +5451,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -5330,10 +5468,10 @@
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>38</v>
@@ -5341,40 +5479,40 @@
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B23" s="26" t="n">
         <v>50665.81</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B24" s="26" t="n">
         <v>210</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B25" s="26" t="n">
         <v>1300</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B26" s="67" t="n">
         <f aca="false">SUM(B23:B25)</f>
@@ -5384,7 +5522,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -5396,112 +5534,112 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5544,22 +5682,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -5568,14 +5706,14 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>38</v>
@@ -5583,74 +5721,74 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="70" t="s">
-        <v>213</v>
+      <c r="D7" s="72" t="s">
+        <v>218</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="8" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="16" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B9" s="7"/>
-      <c r="C9" s="72" t="n">
+      <c r="C9" s="74" t="n">
         <v>350000</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="16" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B10" s="7"/>
-      <c r="C10" s="72" t="n">
+      <c r="C10" s="74" t="n">
         <v>24000</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="16" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="8" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="16" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="13" t="n">
@@ -5660,12 +5798,12 @@
         <v>0.03</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="13" t="n">
@@ -5675,12 +5813,12 @@
         <v>0.02</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="13" t="n">
@@ -5688,12 +5826,12 @@
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="16" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -5710,31 +5848,31 @@
         <v>34</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5766,11 +5904,11 @@
         <f aca="false">IF($C19&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I19" s="73" t="n">
+      <c r="I19" s="75" t="n">
         <f aca="false">IF($C19&lt;&gt;"Yes",0,MIN($B19,$C$9)*($C$13*MIN($D19,$D$13)+$C$14*MIN(MAX($D19-$D$13,0),$D$14)))</f>
         <v>7440</v>
       </c>
-      <c r="J19" s="73" t="n">
+      <c r="J19" s="75" t="n">
         <f aca="false">IF($C19&lt;&gt;"Yes",0,MIN($B19,$C$9)*$C$15)</f>
         <v>5580</v>
       </c>
@@ -5804,11 +5942,11 @@
         <f aca="false">IF($C20&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I20" s="73" t="n">
+      <c r="I20" s="75" t="n">
         <f aca="false">IF($C20&lt;&gt;"Yes",0,MIN($B20,$C$9)*($C$13*MIN($D20,$D$13)+$C$14*MIN(MAX($D20-$D$13,0),$D$14)))</f>
         <v>7123.76</v>
       </c>
-      <c r="J20" s="73" t="n">
+      <c r="J20" s="75" t="n">
         <f aca="false">IF($C20&lt;&gt;"Yes",0,MIN($B20,$C$9)*$C$15)</f>
         <v>5342.82</v>
       </c>
@@ -5842,11 +5980,11 @@
         <f aca="false">IF($C21&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I21" s="73" t="n">
+      <c r="I21" s="75" t="n">
         <f aca="false">IF($C21&lt;&gt;"Yes",0,MIN($B21,$C$9)*($C$13*MIN($D21,$D$13)+$C$14*MIN(MAX($D21-$D$13,0),$D$14)))</f>
         <v>5400</v>
       </c>
-      <c r="J21" s="73" t="n">
+      <c r="J21" s="75" t="n">
         <f aca="false">IF($C21&lt;&gt;"Yes",0,MIN($B21,$C$9)*$C$15)</f>
         <v>4050</v>
       </c>
@@ -5880,11 +6018,11 @@
         <f aca="false">IF($C22&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I22" s="73" t="n">
+      <c r="I22" s="75" t="n">
         <f aca="false">IF($C22&lt;&gt;"Yes",0,MIN($B22,$C$9)*($C$13*MIN($D22,$D$13)+$C$14*MIN(MAX($D22-$D$13,0),$D$14)))</f>
         <v>3169.12</v>
       </c>
-      <c r="J22" s="73" t="n">
+      <c r="J22" s="75" t="n">
         <f aca="false">IF($C22&lt;&gt;"Yes",0,MIN($B22,$C$9)*$C$15)</f>
         <v>2376.84</v>
       </c>
@@ -5918,11 +6056,11 @@
         <f aca="false">IF($C23&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I23" s="73" t="n">
+      <c r="I23" s="75" t="n">
         <f aca="false">IF($C23&lt;&gt;"Yes",0,MIN($B23,$C$9)*($C$13*MIN($D23,$D$13)+$C$14*MIN(MAX($D23-$D$13,0),$D$14)))</f>
         <v>3200</v>
       </c>
-      <c r="J23" s="73" t="n">
+      <c r="J23" s="75" t="n">
         <f aca="false">IF($C23&lt;&gt;"Yes",0,MIN($B23,$C$9)*$C$15)</f>
         <v>2400</v>
       </c>
@@ -5948,7 +6086,7 @@
         <f aca="false">SUM(F19:F23)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="74" t="n">
+      <c r="G24" s="76" t="n">
         <f aca="false">IF(B24=0,0,F24/B24)</f>
         <v>0</v>
       </c>
@@ -5967,12 +6105,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -5982,21 +6120,21 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B29" s="50" t="n">
         <v>0</v>
@@ -6006,12 +6144,12 @@
         <v>0</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B30" s="50" t="n">
         <f aca="false">I24</f>
@@ -6022,12 +6160,12 @@
         <v>2194.40666666667</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">J24</f>
@@ -6038,12 +6176,12 @@
         <v>1645.805</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -6052,13 +6190,13 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>38</v>
@@ -6066,7 +6204,7 @@
     </row>
     <row r="35" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B35" s="47" t="n">
         <f aca="false">C35/12</f>
@@ -6077,12 +6215,12 @@
         <v>0</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B36" s="47" t="n">
         <f aca="false">C36/12</f>
@@ -6093,12 +6231,12 @@
         <v>0</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B37" s="66" t="n">
         <f aca="false">SUM(B35:B36)</f>
@@ -6112,7 +6250,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -6120,38 +6258,38 @@
       <c r="E39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="75" t="s">
-        <v>261</v>
+      <c r="A40" s="77" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="75" t="s">
-        <v>262</v>
+      <c r="A41" s="77" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="75" t="s">
-        <v>263</v>
+      <c r="A42" s="77" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="75" t="s">
-        <v>264</v>
+      <c r="A43" s="77" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="75" t="s">
-        <v>265</v>
+      <c r="A44" s="77" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="75" t="s">
-        <v>266</v>
+      <c r="A45" s="77" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="75" t="s">
-        <v>267</v>
+      <c r="A46" s="77" t="s">
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -6195,17 +6333,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -6215,16 +6353,16 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>38</v>
@@ -6232,10 +6370,10 @@
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="B7" s="70" t="s">
-        <v>273</v>
+        <v>277</v>
+      </c>
+      <c r="B7" s="72" t="s">
+        <v>278</v>
       </c>
       <c r="C7" s="47" t="n">
         <f aca="false">Elections!$H$12</f>
@@ -6246,15 +6384,15 @@
         <v>24498</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B8" s="70" t="s">
-        <v>275</v>
+        <v>143</v>
+      </c>
+      <c r="B8" s="72" t="s">
+        <v>280</v>
       </c>
       <c r="C8" s="47" t="n">
         <f aca="false">Questco!F6</f>
@@ -6265,15 +6403,15 @@
         <v>7020</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="B9" s="70" t="s">
-        <v>275</v>
+        <v>282</v>
+      </c>
+      <c r="B9" s="72" t="s">
+        <v>280</v>
       </c>
       <c r="C9" s="47" t="n">
         <f aca="false">Questco!F7</f>
@@ -6284,15 +6422,15 @@
         <v>1402.13</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B10" s="70" t="s">
-        <v>275</v>
+        <v>150</v>
+      </c>
+      <c r="B10" s="72" t="s">
+        <v>280</v>
       </c>
       <c r="C10" s="47" t="n">
         <f aca="false">Questco!F8</f>
@@ -6303,15 +6441,15 @@
         <v>0</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" s="72" t="s">
         <v>280</v>
-      </c>
-      <c r="B11" s="70" t="s">
-        <v>275</v>
       </c>
       <c r="C11" s="47" t="n">
         <f aca="false">Questco!D18</f>
@@ -6322,15 +6460,15 @@
         <v>2464.08</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="B12" s="70" t="s">
-        <v>275</v>
+        <v>287</v>
+      </c>
+      <c r="B12" s="72" t="s">
+        <v>280</v>
       </c>
       <c r="C12" s="47" t="n">
         <f aca="false">'401(k)'!B37</f>
@@ -6341,12 +6479,12 @@
         <v>0</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="66" t="n">
@@ -6361,10 +6499,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="B14" s="70" t="s">
-        <v>275</v>
+        <v>290</v>
+      </c>
+      <c r="B14" s="72" t="s">
+        <v>280</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="25" t="n">
@@ -6375,7 +6513,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="66" t="n">
@@ -6389,23 +6527,23 @@
       <c r="E15" s="33"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="76" t="s">
-        <v>287</v>
+      <c r="A16" s="78" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="45" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -6415,13 +6553,13 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>38</v>
@@ -6429,7 +6567,7 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B22" s="47" t="n">
         <f aca="false">Elections!$I$12</f>
@@ -6440,12 +6578,12 @@
         <v>24498</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B23" s="47" t="n">
         <f aca="false">'401(k)'!E24/12</f>
@@ -6456,12 +6594,12 @@
         <v>39499.32</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B24" s="47" t="n">
         <f aca="false">IF('401(k)'!$C$8="Employer",0,'401(k)'!H24/12)</f>
@@ -6472,12 +6610,12 @@
         <v>60</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B25" s="24" t="n">
         <f aca="false">Elections!$J$12</f>
@@ -6488,12 +6626,12 @@
         <v>48996</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B26" s="24" t="n">
         <f aca="false">C13+B22+B24</f>
@@ -6504,25 +6642,25 @@
         <v>59942.21</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="50" t="n">
-        <f aca="false">D13+SUMPRODUCT(('Cost by Tier'!$A$5:$A$16=Elections!$E$7)*'Cost by Tier'!$S$5:$S$16*'Cost by Tier'!$E$5:$E$16)</f>
+        <f aca="false">D13+SUMPRODUCT(('Cost by Tier'!$A$5:$A$21=Elections!$E$7)*'Cost by Tier'!$S$5:$S$21*'Cost by Tier'!$E$5:$E$21)</f>
         <v>94882.21</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -6533,25 +6671,25 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>56</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6562,7 +6700,7 @@
         <v>67</v>
       </c>
       <c r="C31" s="25" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$16,'Cost by Tier'!$A$5:$A$16,$A31)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$21,'Cost by Tier'!$A$5:$A$21,$A31)</f>
         <v>24498</v>
       </c>
       <c r="D31" s="50" t="n">
@@ -6570,7 +6708,7 @@
         <v>35384.21</v>
       </c>
       <c r="E31" s="25" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$16,'Cost by Tier'!$A$5:$A$16,$A31)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$21,'Cost by Tier'!$A$5:$A$21,$A31)</f>
         <v>24498</v>
       </c>
       <c r="F31" s="25" t="n">
@@ -6578,7 +6716,7 @@
         <v>59942.21</v>
       </c>
       <c r="G31" s="25" t="n">
-        <f aca="false">D31+SUMPRODUCT(('Cost by Tier'!$A$5:$A$16=$A31)*'Cost by Tier'!$S$5:$S$16*'Cost by Tier'!$E$5:$E$16)</f>
+        <f aca="false">D31+SUMPRODUCT(('Cost by Tier'!$A$5:$A$21=$A31)*'Cost by Tier'!$S$5:$S$21*'Cost by Tier'!$E$5:$E$21)</f>
         <v>94882.21</v>
       </c>
     </row>
@@ -6590,7 +6728,7 @@
         <v>72</v>
       </c>
       <c r="C32" s="58" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$16,'Cost by Tier'!$A$5:$A$16,$A32)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$21,'Cost by Tier'!$A$5:$A$21,$A32)</f>
         <v>27459.72</v>
       </c>
       <c r="D32" s="60" t="n">
@@ -6598,7 +6736,7 @@
         <v>38345.93</v>
       </c>
       <c r="E32" s="58" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$16,'Cost by Tier'!$A$5:$A$16,$A32)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$21,'Cost by Tier'!$A$5:$A$21,$A32)</f>
         <v>27459.72</v>
       </c>
       <c r="F32" s="58" t="n">
@@ -6606,7 +6744,7 @@
         <v>65865.65</v>
       </c>
       <c r="G32" s="58" t="n">
-        <f aca="false">D32+SUMPRODUCT(('Cost by Tier'!$A$5:$A$16=$A32)*'Cost by Tier'!$S$5:$S$16*'Cost by Tier'!$E$5:$E$16)</f>
+        <f aca="false">D32+SUMPRODUCT(('Cost by Tier'!$A$5:$A$21=$A32)*'Cost by Tier'!$S$5:$S$21*'Cost by Tier'!$E$5:$E$21)</f>
         <v>93805.65</v>
       </c>
     </row>
@@ -6618,7 +6756,7 @@
         <v>72</v>
       </c>
       <c r="C33" s="25" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$16,'Cost by Tier'!$A$5:$A$16,$A33)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$M$5:$M$21,'Cost by Tier'!$A$5:$A$21,$A33)</f>
         <v>30485.04</v>
       </c>
       <c r="D33" s="50" t="n">
@@ -6626,7 +6764,7 @@
         <v>41371.25</v>
       </c>
       <c r="E33" s="25" t="n">
-        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$16,'Cost by Tier'!$A$5:$A$16,$A33)</f>
+        <f aca="false">SUMIFS('Cost by Tier'!$O$5:$O$21,'Cost by Tier'!$A$5:$A$21,$A33)</f>
         <v>30485.04</v>
       </c>
       <c r="F33" s="25" t="n">
@@ -6634,18 +6772,18 @@
         <v>71916.29</v>
       </c>
       <c r="G33" s="25" t="n">
-        <f aca="false">D33+SUMPRODUCT(('Cost by Tier'!$A$5:$A$16=$A33)*'Cost by Tier'!$S$5:$S$16*'Cost by Tier'!$E$5:$E$16)</f>
+        <f aca="false">D33+SUMPRODUCT(('Cost by Tier'!$A$5:$A$21=$A33)*'Cost by Tier'!$S$5:$S$21*'Cost by Tier'!$E$5:$E$21)</f>
         <v>85856.29</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Elections: saved scenario columns for comparing contribution rates
Four named scenario columns below the elections table. Each holds a
percentage per person and reports Onyx monthly and annual, the
employees' side, and the change against Scenario 1.

Columns 1 and 2 ship filled in as a worked example - everyone at 50%
against Christine at 55% - and columns 3 and 4 are blank slots.

It is a scratchpad: it reads each person's plan, tier and enrolment
from the table above and feeds nothing, so the Combined tab is
unaffected by anything typed here. Angle's minimum funding still
floors each figure.

618 formulas, zero errors. The scenario grid was checked against an
independent recomputation under edited percentages, mixed plan
elections, and a rate low enough to hit the Angle floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E1Hoi5T9BmzS6cxcPMES4F
</commit_message>
<xml_diff>
--- a/deliverables/Onyx_Angle_Questco_Cost_Model.xlsx
+++ b/deliverables/Onyx_Angle_Questco_Cost_Model.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="331">
   <si>
     <t xml:space="preserve">Onyx Accounting Group, LLC - Angle Health + Questco</t>
   </si>
@@ -418,6 +418,48 @@
   </si>
   <si>
     <t xml:space="preserve">Everyone defaults to the HDHP 3400/5000. Change the ELECTED PLAN cells as people choose; nothing else needs touching.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAVED SCENARIOS   &lt;- name a column, type a percentage for each person, read the totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A scratchpad. Nothing here feeds the Combined tab - it is only for comparing. Everyone's plan, tier and enrolment come from the table above, so the only thing that changes between columns is the percentage Onyx funds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.  Current - 50% all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.  Christine at 55%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.  (name this one)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.  (name this one)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elected plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium $/mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onyx %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change to ONYX $/yr vs Scenario 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change to employees $/yr vs Scenario 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onyx never pays less than Angle's minimum funding, so a percentage low enough to fall under it gets topped up automatically - which is why the totals stop falling below a floor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario 1 is the baseline the two change rows measure against. Overwrite any column's name and percentages to try something else.</t>
   </si>
   <si>
     <t xml:space="preserve">Every Angle plan, priced for each person</t>
@@ -1244,7 +1286,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="84">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1522,6 +1564,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3871,13 +3933,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
@@ -4304,7 +4366,507 @@
         <v>128</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="E25" s="71" t="s">
+        <v>132</v>
+      </c>
+      <c r="F25" s="71"/>
+      <c r="G25" s="71" t="s">
+        <v>133</v>
+      </c>
+      <c r="H25" s="71"/>
+      <c r="I25" s="71" t="s">
+        <v>134</v>
+      </c>
+      <c r="J25" s="71"/>
+      <c r="K25" s="71" t="s">
+        <v>135</v>
+      </c>
+      <c r="L25" s="71"/>
+    </row>
+    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="K26" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="72" t="str">
+        <f aca="false">$A$7</f>
+        <v>Steven Nikolov</v>
+      </c>
+      <c r="B27" s="28" t="str">
+        <f aca="false">$D$7</f>
+        <v>FAM</v>
+      </c>
+      <c r="C27" s="72" t="str">
+        <f aca="false">$E$7</f>
+        <v>ANG HDHP 3400/5000</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">$G$7</f>
+        <v>1361</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F27" s="47" t="n">
+        <f aca="false">IF(OR($B$7&lt;&gt;"Yes",$F$7&lt;&gt;"Yes"),0,MIN($D27,MAX(E27*$D27,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="G27" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H27" s="47" t="n">
+        <f aca="false">IF(OR($B$7&lt;&gt;"Yes",$F$7&lt;&gt;"Yes"),0,MIN($D27,MAX(G27*$D27,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="I27" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J27" s="47" t="n">
+        <f aca="false">IF(OR($B$7&lt;&gt;"Yes",$F$7&lt;&gt;"Yes"),0,MIN($D27,MAX(I27*$D27,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="K27" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L27" s="47" t="n">
+        <f aca="false">IF(OR($B$7&lt;&gt;"Yes",$F$7&lt;&gt;"Yes"),0,MIN($D27,MAX(K27*$D27,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="72" t="str">
+        <f aca="false">$A$8</f>
+        <v>Lisa Danforth</v>
+      </c>
+      <c r="B28" s="28" t="str">
+        <f aca="false">$D$8</f>
+        <v>EE</v>
+      </c>
+      <c r="C28" s="72" t="str">
+        <f aca="false">$E$8</f>
+        <v>ANG HDHP 3400/5000</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <f aca="false">$G$8</f>
+        <v>439.03</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F28" s="47" t="n">
+        <f aca="false">IF(OR($B$8&lt;&gt;"Yes",$F$8&lt;&gt;"Yes"),0,MIN($D28,MAX(E28*$D28,Contributions!$C$20)))</f>
+        <v>219.515</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H28" s="47" t="n">
+        <f aca="false">IF(OR($B$8&lt;&gt;"Yes",$F$8&lt;&gt;"Yes"),0,MIN($D28,MAX(G28*$D28,Contributions!$C$20)))</f>
+        <v>219.515</v>
+      </c>
+      <c r="I28" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J28" s="47" t="n">
+        <f aca="false">IF(OR($B$8&lt;&gt;"Yes",$F$8&lt;&gt;"Yes"),0,MIN($D28,MAX(I28*$D28,Contributions!$C$20)))</f>
+        <v>219.515</v>
+      </c>
+      <c r="K28" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L28" s="47" t="n">
+        <f aca="false">IF(OR($B$8&lt;&gt;"Yes",$F$8&lt;&gt;"Yes"),0,MIN($D28,MAX(K28*$D28,Contributions!$C$20)))</f>
+        <v>219.515</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="72" t="str">
+        <f aca="false">$A$9</f>
+        <v>Jessica Bumphus</v>
+      </c>
+      <c r="B29" s="28" t="str">
+        <f aca="false">$D$9</f>
+        <v>FAM</v>
+      </c>
+      <c r="C29" s="72" t="str">
+        <f aca="false">$E$9</f>
+        <v>ANG HDHP 3400/5000</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <f aca="false">$G$9</f>
+        <v>1361</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F29" s="47" t="n">
+        <f aca="false">IF(OR($B$9&lt;&gt;"Yes",$F$9&lt;&gt;"Yes"),0,MIN($D29,MAX(E29*$D29,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H29" s="47" t="n">
+        <f aca="false">IF(OR($B$9&lt;&gt;"Yes",$F$9&lt;&gt;"Yes"),0,MIN($D29,MAX(G29*$D29,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="I29" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J29" s="47" t="n">
+        <f aca="false">IF(OR($B$9&lt;&gt;"Yes",$F$9&lt;&gt;"Yes"),0,MIN($D29,MAX(I29*$D29,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+      <c r="K29" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L29" s="47" t="n">
+        <f aca="false">IF(OR($B$9&lt;&gt;"Yes",$F$9&lt;&gt;"Yes"),0,MIN($D29,MAX(K29*$D29,Contributions!$C$20)))</f>
+        <v>680.5</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="72" t="str">
+        <f aca="false">$A$10</f>
+        <v>Christine Johnson</v>
+      </c>
+      <c r="B30" s="28" t="str">
+        <f aca="false">$D$10</f>
+        <v>ES</v>
+      </c>
+      <c r="C30" s="72" t="str">
+        <f aca="false">$E$10</f>
+        <v>ANG HDHP 3400/5000</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <f aca="false">$G$10</f>
+        <v>921.97</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F30" s="47" t="n">
+        <f aca="false">IF(OR($B$10&lt;&gt;"Yes",$F$10&lt;&gt;"Yes"),0,MIN($D30,MAX(E30*$D30,Contributions!$C$20)))</f>
+        <v>460.985</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H30" s="47" t="n">
+        <f aca="false">IF(OR($B$10&lt;&gt;"Yes",$F$10&lt;&gt;"Yes"),0,MIN($D30,MAX(G30*$D30,Contributions!$C$20)))</f>
+        <v>507.0835</v>
+      </c>
+      <c r="I30" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J30" s="47" t="n">
+        <f aca="false">IF(OR($B$10&lt;&gt;"Yes",$F$10&lt;&gt;"Yes"),0,MIN($D30,MAX(I30*$D30,Contributions!$C$20)))</f>
+        <v>460.985</v>
+      </c>
+      <c r="K30" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L30" s="47" t="n">
+        <f aca="false">IF(OR($B$10&lt;&gt;"Yes",$F$10&lt;&gt;"Yes"),0,MIN($D30,MAX(K30*$D30,Contributions!$C$20)))</f>
+        <v>460.985</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="73" t="str">
+        <f aca="false">$A$11</f>
+        <v>Josephine Mack</v>
+      </c>
+      <c r="B31" s="54" t="str">
+        <f aca="false">$D$11</f>
+        <v>FAM</v>
+      </c>
+      <c r="C31" s="73" t="str">
+        <f aca="false">$E$11</f>
+        <v>ANG HDHP 3400/5000</v>
+      </c>
+      <c r="D31" s="55" t="n">
+        <f aca="false">$G$11</f>
+        <v>1361</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F31" s="56" t="n">
+        <f aca="false">IF(OR($B$11&lt;&gt;"Yes",$F$11&lt;&gt;"Yes"),0,MIN($D31,MAX(E31*$D31,Contributions!$C$20)))</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H31" s="56" t="n">
+        <f aca="false">IF(OR($B$11&lt;&gt;"Yes",$F$11&lt;&gt;"Yes"),0,MIN($D31,MAX(G31*$D31,Contributions!$C$20)))</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J31" s="56" t="n">
+        <f aca="false">IF(OR($B$11&lt;&gt;"Yes",$F$11&lt;&gt;"Yes"),0,MIN($D31,MAX(I31*$D31,Contributions!$C$20)))</f>
+        <v>0</v>
+      </c>
+      <c r="K31" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L31" s="56" t="n">
+        <f aca="false">IF(OR($B$11&lt;&gt;"Yes",$F$11&lt;&gt;"Yes"),0,MIN($D31,MAX(K31*$D31,Contributions!$C$20)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="66" t="n">
+        <f aca="false">SUM(F27:F31)</f>
+        <v>2041.5</v>
+      </c>
+      <c r="G32" s="33"/>
+      <c r="H32" s="66" t="n">
+        <f aca="false">SUM(H27:H31)</f>
+        <v>2087.5985</v>
+      </c>
+      <c r="I32" s="33"/>
+      <c r="J32" s="66" t="n">
+        <f aca="false">SUM(J27:J31)</f>
+        <v>2041.5</v>
+      </c>
+      <c r="K32" s="33"/>
+      <c r="L32" s="66" t="n">
+        <f aca="false">SUM(L27:L31)</f>
+        <v>2041.5</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="B33" s="33"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="67" t="n">
+        <f aca="false">F32*12</f>
+        <v>24498</v>
+      </c>
+      <c r="G33" s="33"/>
+      <c r="H33" s="67" t="n">
+        <f aca="false">H32*12</f>
+        <v>25051.182</v>
+      </c>
+      <c r="I33" s="33"/>
+      <c r="J33" s="67" t="n">
+        <f aca="false">J32*12</f>
+        <v>24498</v>
+      </c>
+      <c r="K33" s="33"/>
+      <c r="L33" s="67" t="n">
+        <f aca="false">L32*12</f>
+        <v>24498</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="47" t="n">
+        <f aca="false">SUMPRODUCT(($B$7:$B$11="Yes")*($F$7:$F$11="Yes")*$G$7:$G$11)-F32</f>
+        <v>2041.5</v>
+      </c>
+      <c r="G34" s="7"/>
+      <c r="H34" s="47" t="n">
+        <f aca="false">SUMPRODUCT(($B$7:$B$11="Yes")*($F$7:$F$11="Yes")*$G$7:$G$11)-H32</f>
+        <v>1995.4015</v>
+      </c>
+      <c r="I34" s="7"/>
+      <c r="J34" s="47" t="n">
+        <f aca="false">SUMPRODUCT(($B$7:$B$11="Yes")*($F$7:$F$11="Yes")*$G$7:$G$11)-J32</f>
+        <v>2041.5</v>
+      </c>
+      <c r="K34" s="7"/>
+      <c r="L34" s="47" t="n">
+        <f aca="false">SUMPRODUCT(($B$7:$B$11="Yes")*($F$7:$F$11="Yes")*$G$7:$G$11)-L32</f>
+        <v>2041.5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="25" t="n">
+        <f aca="false">F34*12</f>
+        <v>24498</v>
+      </c>
+      <c r="G35" s="7"/>
+      <c r="H35" s="25" t="n">
+        <f aca="false">H34*12</f>
+        <v>23944.818</v>
+      </c>
+      <c r="I35" s="7"/>
+      <c r="J35" s="25" t="n">
+        <f aca="false">J34*12</f>
+        <v>24498</v>
+      </c>
+      <c r="K35" s="7"/>
+      <c r="L35" s="25" t="n">
+        <f aca="false">L34*12</f>
+        <v>24498</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="67" t="n">
+        <f aca="false">F33-$F$33</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="33"/>
+      <c r="H36" s="67" t="n">
+        <f aca="false">H33-$F$33</f>
+        <v>553.182000000001</v>
+      </c>
+      <c r="I36" s="33"/>
+      <c r="J36" s="67" t="n">
+        <f aca="false">J33-$F$33</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="33"/>
+      <c r="L36" s="67" t="n">
+        <f aca="false">L33-$F$33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="25" t="n">
+        <f aca="false">F35-$F$35</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="7"/>
+      <c r="H37" s="25" t="n">
+        <f aca="false">H35-$F$35</f>
+        <v>-553.182000000001</v>
+      </c>
+      <c r="I37" s="7"/>
+      <c r="J37" s="25" t="n">
+        <f aca="false">J35-$F$35</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="7"/>
+      <c r="L37" s="25" t="n">
+        <f aca="false">L35-$F$35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="74" t="str">
+        <f aca="false">IF($H$36=0,"Scenario 2 costs Onyx exactly what Scenario 1 does.","Scenario 2 costs Onyx "&amp;TEXT(ABS($H$36),"$#,##0")&amp;IF($H$36&gt;0," MORE"," LESS")&amp;" a year than Scenario 1 - and moves that same amount "&amp;IF($H$36&gt;0,"off","onto")&amp;" the employees.")</f>
+        <v>Scenario 2 costs Onyx $553 MORE a year than Scenario 1 - and moves that same amount off the employees.</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="K25:L25"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E7:E11" type="list">
       <formula1>"ANG HDHP 3400/5000,ANG TRAD 2000/4000,ANG TRAD 1000/2000"</formula1>
@@ -4342,12 +4904,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4373,7 +4935,7 @@
         <v>90</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>117</v>
@@ -4388,7 +4950,7 @@
         <v>101</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4436,7 +4998,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M5" s="70" t="n">
+      <c r="M5" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E5&amp;"|"&amp;$D5,CostKey,0))</f>
         <v>18166</v>
       </c>
@@ -4486,7 +5048,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M6" s="70" t="n">
+      <c r="M6" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E6&amp;"|"&amp;$D6,CostKey,0))</f>
         <v>17153.24</v>
       </c>
@@ -4536,7 +5098,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M7" s="70" t="n">
+      <c r="M7" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E7&amp;"|"&amp;$D7,CostKey,0))</f>
         <v>14161.66</v>
       </c>
@@ -4586,7 +5148,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>5000</v>
       </c>
-      <c r="M8" s="70" t="n">
+      <c r="M8" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E8&amp;"|"&amp;$D8,CostKey,0))</f>
         <v>7634.18</v>
       </c>
@@ -4636,7 +5198,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M9" s="70" t="n">
+      <c r="M9" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E9&amp;"|"&amp;$D9,CostKey,0))</f>
         <v>6952.66</v>
       </c>
@@ -4686,7 +5248,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>2000</v>
       </c>
-      <c r="M10" s="70" t="n">
+      <c r="M10" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E10&amp;"|"&amp;$D10,CostKey,0))</f>
         <v>5277.98</v>
       </c>
@@ -4736,7 +5298,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M11" s="70" t="n">
+      <c r="M11" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E11&amp;"|"&amp;$D11,CostKey,0))</f>
         <v>18166</v>
       </c>
@@ -4786,7 +5348,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M12" s="70" t="n">
+      <c r="M12" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E12&amp;"|"&amp;$D12,CostKey,0))</f>
         <v>17153.24</v>
       </c>
@@ -4836,7 +5398,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M13" s="70" t="n">
+      <c r="M13" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E13&amp;"|"&amp;$D13,CostKey,0))</f>
         <v>14161.66</v>
       </c>
@@ -4886,7 +5448,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M14" s="70" t="n">
+      <c r="M14" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E14&amp;"|"&amp;$D14,CostKey,0))</f>
         <v>15531.82</v>
       </c>
@@ -4936,7 +5498,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M15" s="70" t="n">
+      <c r="M15" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E15&amp;"|"&amp;$D15,CostKey,0))</f>
         <v>14200.58</v>
       </c>
@@ -4986,7 +5548,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M16" s="70" t="n">
+      <c r="M16" s="75" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E16&amp;"|"&amp;$D16,CostKey,0))</f>
         <v>10883.74</v>
       </c>
@@ -5036,7 +5598,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>10000</v>
       </c>
-      <c r="M17" s="71" t="n">
+      <c r="M17" s="76" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E17&amp;"|"&amp;$D17,CostKey,0))</f>
         <v>18166</v>
       </c>
@@ -5086,7 +5648,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>8000</v>
       </c>
-      <c r="M18" s="71" t="n">
+      <c r="M18" s="76" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E18&amp;"|"&amp;$D18,CostKey,0))</f>
         <v>17153.24</v>
       </c>
@@ -5136,7 +5698,7 @@
         <f aca="false">INDEX('Cost by Tier'!$R$5:$R$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>4000</v>
       </c>
-      <c r="M19" s="71" t="n">
+      <c r="M19" s="76" t="n">
         <f aca="false">INDEX('Cost by Tier'!$S$5:$S$21,MATCH($E19&amp;"|"&amp;$D19,CostKey,0))</f>
         <v>14161.66</v>
       </c>
@@ -5173,17 +5735,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -5195,25 +5757,25 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>38</v>
@@ -5221,10 +5783,10 @@
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" s="72" t="s">
-        <v>144</v>
+        <v>157</v>
+      </c>
+      <c r="B6" s="77" t="s">
+        <v>158</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>117</v>
@@ -5232,8 +5794,8 @@
       <c r="D6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="73" t="s">
-        <v>145</v>
+      <c r="E6" s="78" t="s">
+        <v>159</v>
       </c>
       <c r="F6" s="47" t="n">
         <f aca="false">G6/12</f>
@@ -5244,22 +5806,22 @@
         <v>7020</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B7" s="72" t="s">
-        <v>148</v>
+        <v>161</v>
+      </c>
+      <c r="B7" s="77" t="s">
+        <v>162</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>1402.13</v>
       </c>
       <c r="D7" s="7"/>
-      <c r="E7" s="73" t="s">
-        <v>145</v>
+      <c r="E7" s="78" t="s">
+        <v>159</v>
       </c>
       <c r="F7" s="47" t="n">
         <f aca="false">G7/12</f>
@@ -5270,15 +5832,15 @@
         <v>1402.13</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B8" s="72" t="s">
-        <v>148</v>
+        <v>164</v>
+      </c>
+      <c r="B8" s="77" t="s">
+        <v>162</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>420</v>
@@ -5296,12 +5858,12 @@
         <v>0</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
@@ -5319,28 +5881,28 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B10" s="72" t="s">
-        <v>154</v>
+        <v>167</v>
+      </c>
+      <c r="B10" s="77" t="s">
+        <v>168</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
-      <c r="G10" s="74" t="n">
+      <c r="G10" s="79" t="n">
         <v>1000</v>
       </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -5352,19 +5914,19 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>38</v>
@@ -5372,13 +5934,13 @@
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="72" t="s">
-        <v>160</v>
+      <c r="C15" s="77" t="s">
+        <v>174</v>
       </c>
       <c r="D15" s="14" t="n">
         <v>46.25</v>
@@ -5388,18 +5950,18 @@
         <v>555</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="72" t="s">
-        <v>163</v>
+      <c r="C16" s="77" t="s">
+        <v>177</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>159.09</v>
@@ -5409,18 +5971,18 @@
         <v>1909.08</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="72" t="s">
-        <v>166</v>
+      <c r="C17" s="77" t="s">
+        <v>180</v>
       </c>
       <c r="D17" s="14" t="n">
         <v>126.74</v>
@@ -5430,12 +5992,12 @@
         <v>0</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B18" s="33"/>
       <c r="C18" s="33"/>
@@ -5451,12 +6013,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -5468,10 +6030,10 @@
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>38</v>
@@ -5479,40 +6041,40 @@
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B23" s="26" t="n">
         <v>50665.81</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B24" s="26" t="n">
         <v>210</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="B25" s="26" t="n">
         <v>1300</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B26" s="67" t="n">
         <f aca="false">SUM(B23:B25)</f>
@@ -5522,7 +6084,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -5534,112 +6096,112 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -5682,22 +6244,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -5706,14 +6268,14 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>38</v>
@@ -5721,74 +6283,74 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="72" t="s">
-        <v>218</v>
+      <c r="D7" s="77" t="s">
+        <v>232</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="8" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="16" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="B9" s="7"/>
-      <c r="C9" s="74" t="n">
+      <c r="C9" s="79" t="n">
         <v>350000</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="16" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="B10" s="7"/>
-      <c r="C10" s="74" t="n">
+      <c r="C10" s="79" t="n">
         <v>24000</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="16" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="8" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="16" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="13" t="n">
@@ -5798,12 +6360,12 @@
         <v>0.03</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="13" t="n">
@@ -5813,12 +6375,12 @@
         <v>0.02</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="13" t="n">
@@ -5826,12 +6388,12 @@
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="16" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -5848,31 +6410,31 @@
         <v>34</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5904,11 +6466,11 @@
         <f aca="false">IF($C19&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I19" s="75" t="n">
+      <c r="I19" s="80" t="n">
         <f aca="false">IF($C19&lt;&gt;"Yes",0,MIN($B19,$C$9)*($C$13*MIN($D19,$D$13)+$C$14*MIN(MAX($D19-$D$13,0),$D$14)))</f>
         <v>7440</v>
       </c>
-      <c r="J19" s="75" t="n">
+      <c r="J19" s="80" t="n">
         <f aca="false">IF($C19&lt;&gt;"Yes",0,MIN($B19,$C$9)*$C$15)</f>
         <v>5580</v>
       </c>
@@ -5942,11 +6504,11 @@
         <f aca="false">IF($C20&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I20" s="75" t="n">
+      <c r="I20" s="80" t="n">
         <f aca="false">IF($C20&lt;&gt;"Yes",0,MIN($B20,$C$9)*($C$13*MIN($D20,$D$13)+$C$14*MIN(MAX($D20-$D$13,0),$D$14)))</f>
         <v>7123.76</v>
       </c>
-      <c r="J20" s="75" t="n">
+      <c r="J20" s="80" t="n">
         <f aca="false">IF($C20&lt;&gt;"Yes",0,MIN($B20,$C$9)*$C$15)</f>
         <v>5342.82</v>
       </c>
@@ -5980,11 +6542,11 @@
         <f aca="false">IF($C21&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I21" s="75" t="n">
+      <c r="I21" s="80" t="n">
         <f aca="false">IF($C21&lt;&gt;"Yes",0,MIN($B21,$C$9)*($C$13*MIN($D21,$D$13)+$C$14*MIN(MAX($D21-$D$13,0),$D$14)))</f>
         <v>5400</v>
       </c>
-      <c r="J21" s="75" t="n">
+      <c r="J21" s="80" t="n">
         <f aca="false">IF($C21&lt;&gt;"Yes",0,MIN($B21,$C$9)*$C$15)</f>
         <v>4050</v>
       </c>
@@ -6018,11 +6580,11 @@
         <f aca="false">IF($C22&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I22" s="75" t="n">
+      <c r="I22" s="80" t="n">
         <f aca="false">IF($C22&lt;&gt;"Yes",0,MIN($B22,$C$9)*($C$13*MIN($D22,$D$13)+$C$14*MIN(MAX($D22-$D$13,0),$D$14)))</f>
         <v>3169.12</v>
       </c>
-      <c r="J22" s="75" t="n">
+      <c r="J22" s="80" t="n">
         <f aca="false">IF($C22&lt;&gt;"Yes",0,MIN($B22,$C$9)*$C$15)</f>
         <v>2376.84</v>
       </c>
@@ -6056,11 +6618,11 @@
         <f aca="false">IF($C23&lt;&gt;"Yes",0,$C$7*4)</f>
         <v>12</v>
       </c>
-      <c r="I23" s="75" t="n">
+      <c r="I23" s="80" t="n">
         <f aca="false">IF($C23&lt;&gt;"Yes",0,MIN($B23,$C$9)*($C$13*MIN($D23,$D$13)+$C$14*MIN(MAX($D23-$D$13,0),$D$14)))</f>
         <v>3200</v>
       </c>
-      <c r="J23" s="75" t="n">
+      <c r="J23" s="80" t="n">
         <f aca="false">IF($C23&lt;&gt;"Yes",0,MIN($B23,$C$9)*$C$15)</f>
         <v>2400</v>
       </c>
@@ -6086,7 +6648,7 @@
         <f aca="false">SUM(F19:F23)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="76" t="n">
+      <c r="G24" s="81" t="n">
         <f aca="false">IF(B24=0,0,F24/B24)</f>
         <v>0</v>
       </c>
@@ -6105,12 +6667,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -6120,21 +6682,21 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="B29" s="50" t="n">
         <v>0</v>
@@ -6144,12 +6706,12 @@
         <v>0</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="B30" s="50" t="n">
         <f aca="false">I24</f>
@@ -6160,12 +6722,12 @@
         <v>2194.40666666667</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B31" s="50" t="n">
         <f aca="false">J24</f>
@@ -6176,12 +6738,12 @@
         <v>1645.805</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -6190,13 +6752,13 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>38</v>
@@ -6204,7 +6766,7 @@
     </row>
     <row r="35" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="B35" s="47" t="n">
         <f aca="false">C35/12</f>
@@ -6215,12 +6777,12 @@
         <v>0</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="B36" s="47" t="n">
         <f aca="false">C36/12</f>
@@ -6231,12 +6793,12 @@
         <v>0</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B37" s="66" t="n">
         <f aca="false">SUM(B35:B36)</f>
@@ -6250,7 +6812,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -6258,38 +6820,38 @@
       <c r="E39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="77" t="s">
-        <v>266</v>
+      <c r="A40" s="82" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="77" t="s">
-        <v>267</v>
+      <c r="A41" s="82" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="77" t="s">
-        <v>268</v>
+      <c r="A42" s="82" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="77" t="s">
-        <v>269</v>
+      <c r="A43" s="82" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="77" t="s">
-        <v>270</v>
+      <c r="A44" s="82" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="77" t="s">
-        <v>271</v>
+      <c r="A45" s="82" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="77" t="s">
-        <v>272</v>
+      <c r="A46" s="82" t="s">
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -6333,17 +6895,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -6353,16 +6915,16 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>38</v>
@@ -6370,10 +6932,10 @@
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="B7" s="72" t="s">
-        <v>278</v>
+        <v>291</v>
+      </c>
+      <c r="B7" s="77" t="s">
+        <v>292</v>
       </c>
       <c r="C7" s="47" t="n">
         <f aca="false">Elections!$H$12</f>
@@ -6384,15 +6946,15 @@
         <v>24498</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B8" s="72" t="s">
-        <v>280</v>
+        <v>157</v>
+      </c>
+      <c r="B8" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C8" s="47" t="n">
         <f aca="false">Questco!F6</f>
@@ -6403,15 +6965,15 @@
         <v>7020</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="B9" s="72" t="s">
-        <v>280</v>
+        <v>296</v>
+      </c>
+      <c r="B9" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C9" s="47" t="n">
         <f aca="false">Questco!F7</f>
@@ -6422,15 +6984,15 @@
         <v>1402.13</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B10" s="72" t="s">
-        <v>280</v>
+        <v>164</v>
+      </c>
+      <c r="B10" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C10" s="47" t="n">
         <f aca="false">Questco!F8</f>
@@ -6441,15 +7003,15 @@
         <v>0</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="B11" s="72" t="s">
-        <v>280</v>
+        <v>299</v>
+      </c>
+      <c r="B11" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C11" s="47" t="n">
         <f aca="false">Questco!D18</f>
@@ -6460,15 +7022,15 @@
         <v>2464.08</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="B12" s="72" t="s">
-        <v>280</v>
+        <v>301</v>
+      </c>
+      <c r="B12" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C12" s="47" t="n">
         <f aca="false">'401(k)'!B37</f>
@@ -6479,12 +7041,12 @@
         <v>0</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="66" t="n">
@@ -6499,10 +7061,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="B14" s="72" t="s">
-        <v>280</v>
+        <v>304</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>294</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="25" t="n">
@@ -6513,7 +7075,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="66" t="n">
@@ -6527,23 +7089,23 @@
       <c r="E15" s="33"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="78" t="s">
-        <v>292</v>
+      <c r="A16" s="83" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="45" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -6553,13 +7115,13 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>38</v>
@@ -6567,7 +7129,7 @@
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="B22" s="47" t="n">
         <f aca="false">Elections!$I$12</f>
@@ -6578,12 +7140,12 @@
         <v>24498</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="B23" s="47" t="n">
         <f aca="false">'401(k)'!E24/12</f>
@@ -6594,12 +7156,12 @@
         <v>39499.32</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
       <c r="B24" s="47" t="n">
         <f aca="false">IF('401(k)'!$C$8="Employer",0,'401(k)'!H24/12)</f>
@@ -6610,12 +7172,12 @@
         <v>60</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="B25" s="24" t="n">
         <f aca="false">Elections!$J$12</f>
@@ -6626,12 +7188,12 @@
         <v>48996</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="B26" s="24" t="n">
         <f aca="false">C13+B22+B24</f>
@@ -6642,12 +7204,12 @@
         <v>59942.21</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>306</v>
+        <v>320</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="50" t="n">
@@ -6655,12 +7217,12 @@
         <v>94882.21</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -6671,25 +7233,25 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>56</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6778,12 +7340,12 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>